<commit_message>
Jour 20 : projet intermédiaire - analyse complète
</commit_message>
<xml_diff>
--- a/jour-19-dashboard-interactif/exercices/Jour_19_Dashboard.xlsx
+++ b/jour-19-dashboard-interactif/exercices/Jour_19_Dashboard.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abdou\OneDrive\Documents\BootcampExcel\excel-bootcamp-30-jours\jour-19-dashboard-interactif\exercices\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D563D66-DA98-4D50-9865-2D8F11E10E25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D568CC99-46D5-4B8C-A6F0-CD3CE80A817B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" firstSheet="1" activeTab="1" xr2:uid="{F9491382-A35F-4402-ACA1-0895E46AB027}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" xr2:uid="{F9491382-A35F-4402-ACA1-0895E46AB027}"/>
   </bookViews>
   <sheets>
-    <sheet name="TCD_Effectifs_Dept" sheetId="3" r:id="rId1"/>
-    <sheet name="Dashboard_RH" sheetId="2" r:id="rId2"/>
+    <sheet name="Dashboard_RH" sheetId="2" r:id="rId1"/>
+    <sheet name="TCD_Effectifs_Dept" sheetId="3" r:id="rId2"/>
     <sheet name="TCD_Salaire_Dept" sheetId="4" r:id="rId3"/>
     <sheet name="TCD_Sexe" sheetId="5" r:id="rId4"/>
     <sheet name="TCD_Ville" sheetId="6" r:id="rId5"/>
@@ -27,7 +27,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="8" r:id="rId7"/>
+    <pivotCache cacheId="0" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -721,9 +721,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
-    <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -738,17 +738,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="16"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="16"/>
-      <color theme="4" tint="-0.499984740745262"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
@@ -758,6 +747,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="17"/>
+      <color theme="4" tint="-0.499984740745262"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -803,7 +799,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -816,232 +812,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="70">
+  <dxfs count="2">
     <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
+      <numFmt numFmtId="165" formatCode="#,##0.0\ &quot;€&quot;"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.0\ &quot;€&quot;"/>
+      <numFmt numFmtId="165" formatCode="#,##0.0\ &quot;€&quot;"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -6252,167 +6040,6 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>661988</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>9526</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>204788</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>4764</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-        <xdr:graphicFrame macro="">
-          <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="3" name="Ville">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{63C10698-21CF-49F8-E977-D0582DA019B7}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGraphicFramePr/>
-          </xdr:nvGraphicFramePr>
-          <xdr:xfrm>
-            <a:off x="0" y="0"/>
-            <a:ext cx="0" cy="0"/>
-          </xdr:xfrm>
-          <a:graphic>
-            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
-              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="Ville"/>
-            </a:graphicData>
-          </a:graphic>
-        </xdr:graphicFrame>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="0" name=""/>
-            <xdr:cNvSpPr>
-              <a:spLocks noTextEdit="1"/>
-            </xdr:cNvSpPr>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="5100638" y="190501"/>
-              <a:ext cx="1828800" cy="2166938"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:solidFill>
-              <a:prstClr val="white"/>
-            </a:solidFill>
-            <a:ln w="1">
-              <a:solidFill>
-                <a:prstClr val="green"/>
-              </a:solidFill>
-            </a:ln>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="fr-FR" sz="1100"/>
-                <a:t>Cette forme représente un segment. Les segments sont pris en charge dans Excel 2010 ou version ultérieure.
-En revanche, si la forme a été modifiée dans une version précédente d’Excel, ou si le classeur a été enregistré dans Excel 2003 ou une version précédente, vous ne pouvez pas utiliser le segment.</a:t>
-              </a:r>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>576263</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>119063</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>14288</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-        <xdr:graphicFrame macro="">
-          <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="4" name="Filiere">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9C5CA092-5C67-6A66-7BB6-97D67AEEF4B9}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGraphicFramePr/>
-          </xdr:nvGraphicFramePr>
-          <xdr:xfrm>
-            <a:off x="0" y="0"/>
-            <a:ext cx="0" cy="0"/>
-          </xdr:xfrm>
-          <a:graphic>
-            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
-              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="Filiere"/>
-            </a:graphicData>
-          </a:graphic>
-        </xdr:graphicFrame>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="0" name=""/>
-            <xdr:cNvSpPr>
-              <a:spLocks noTextEdit="1"/>
-            </xdr:cNvSpPr>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="7300913" y="228600"/>
-              <a:ext cx="1828800" cy="1776413"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:solidFill>
-              <a:prstClr val="white"/>
-            </a:solidFill>
-            <a:ln w="1">
-              <a:solidFill>
-                <a:prstClr val="green"/>
-              </a:solidFill>
-            </a:ln>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="fr-FR" sz="1100"/>
-                <a:t>Cette forme représente un segment. Les segments sont pris en charge dans Excel 2010 ou version ultérieure.
-En revanche, si la forme a été modifiée dans une version précédente d’Excel, ou si le classeur a été enregistré dans Excel 2003 ou une version précédente, vous ne pouvez pas utiliser le segment.</a:t>
-              </a:r>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>428625</xdr:colOff>
       <xdr:row>7</xdr:row>
@@ -6422,10 +6049,10 @@
       <xdr:col>7</xdr:col>
       <xdr:colOff>23812</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>104775</xdr:rowOff>
+      <xdr:rowOff>104774</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="4" name="Sexe">
@@ -6448,7 +6075,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -6458,8 +6085,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="3751427" y="1393551"/>
-              <a:ext cx="1877902" cy="955621"/>
+              <a:off x="3747492" y="1384400"/>
+              <a:ext cx="1872258" cy="945356"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -6502,8 +6129,8 @@
       <xdr:row>18</xdr:row>
       <xdr:rowOff>109538</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="5" name="Ville 1">
@@ -6526,7 +6153,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -6536,8 +6163,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="0" y="1374501"/>
-              <a:ext cx="1683024" cy="2063313"/>
+              <a:off x="0" y="1365350"/>
+              <a:ext cx="1684735" cy="2040732"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -6580,8 +6207,8 @@
       <xdr:row>15</xdr:row>
       <xdr:rowOff>100013</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="6" name="Filiere 1">
@@ -6604,7 +6231,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -6614,8 +6241,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="1862905" y="1374502"/>
-              <a:ext cx="1826610" cy="1511848"/>
+              <a:off x="1862733" y="1365351"/>
+              <a:ext cx="1822847" cy="1495425"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -8258,7 +7885,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F693E67B-A3BE-4C0C-B05E-C7EA1A0462F4}" name="Tableau croisé dynamique1" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F693E67B-A3BE-4C0C-B05E-C7EA1A0462F4}" name="Tableau croisé dynamique1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -8337,7 +7964,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3DF99934-89F6-4863-A675-A89847D0D585}" name="Tableau croisé dynamique2" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="12">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3DF99934-89F6-4863-A675-A89847D0D585}" name="Tableau croisé dynamique2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="12">
   <location ref="A3:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField showAll="0"/>
@@ -8401,36 +8028,18 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Moyenne de Frais_payes" fld="10" subtotal="average" baseField="4" baseItem="0" numFmtId="168"/>
+    <dataField name="Moyenne de Frais_payes" fld="10" subtotal="average" baseField="4" baseItem="0" numFmtId="165"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="66">
+    <format dxfId="1">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="67">
+    <format dxfId="0">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
-  <chartFormats count="4">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
+  <chartFormats count="2">
     <chartFormat chart="6" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="7" format="0" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -8462,7 +8071,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7449DC11-A568-4024-857C-3F92FBF591AA}" name="Tableau croisé dynamique3" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7449DC11-A568-4024-857C-3F92FBF591AA}" name="Tableau croisé dynamique3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
   <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -8522,16 +8131,7 @@
   <dataFields count="1">
     <dataField name="Nombre de ID" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
-  <chartFormats count="4">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
+  <chartFormats count="3">
     <chartFormat chart="6" format="4" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
@@ -8579,7 +8179,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F67DEEBB-7CB5-434E-B619-A964373630DC}" name="Tableau croisé dynamique4" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F67DEEBB-7CB5-434E-B619-A964373630DC}" name="Tableau croisé dynamique4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
   <location ref="A3:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -8651,16 +8251,7 @@
   <dataFields count="1">
     <dataField name="Nombre de ID" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
-  <chartFormats count="2">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
+  <chartFormats count="1">
     <chartFormat chart="4" format="2" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
@@ -8747,13 +8338,6 @@
 </file>
 
 <file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
-<slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <slicer name="Ville" xr10:uid="{DE784BD6-E3FC-4764-86BF-21FC94D9B70F}" cache="Segment_Ville1" caption="Ville" rowHeight="249238"/>
-  <slicer name="Filiere" xr10:uid="{DA91FF38-677D-4F0B-BEF4-04ACD76E270E}" cache="Segment_Filiere1" caption="Filiere" rowHeight="249238"/>
-</slicers>
-</file>
-
-<file path=xl/slicers/slicer2.xml><?xml version="1.0" encoding="utf-8"?>
 <slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
   <slicer name="Sexe" xr10:uid="{220AD01A-DED0-408A-8A87-CC36E00CEEB2}" cache="Segment_Sexe" caption="Sexe" rowHeight="249238"/>
   <slicer name="Ville 1" xr10:uid="{5996F2EC-EF70-4BAB-8060-4C687F52E53D}" cache="Segment_Ville1" caption="Ville" rowHeight="249238"/>
@@ -9077,132 +8661,67 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BECCEC7-2499-4969-8C4A-4F59A08AA981}">
-  <dimension ref="A3:B8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="1" max="1" width="18.53125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.59765625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A3" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="B3" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A4" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="B4" s="6">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A5" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="6">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A6" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B6" s="6">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A7" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="6">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A8" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="B8" s="6">
-        <v>99</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId2"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{A8765BA9-456A-4dab-B4F3-ACF838C121DE}">
-      <x14:slicerList>
-        <x14:slicer r:id="rId3"/>
-      </x14:slicerList>
-    </ext>
-  </extLst>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B14EC9C9-8D39-4308-9BB2-B47825E07CF4}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="14.53125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="20.25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A3" s="11" t="s">
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A3" s="8" t="s">
         <v>210</v>
       </c>
-      <c r="B3" s="12">
-        <f>COUNTA(Employes!B:B)-1</f>
+      <c r="B3" s="9">
+        <f>_xlfn.AGGREGATE(3,5,Employes!B:B)-1</f>
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A4" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="10">
         <f>AVERAGE(Employes!K:K)</f>
         <v>86717.171717171717</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A5" s="11" t="s">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A5" s="8" t="s">
         <v>213</v>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="9">
         <f>MAX(Employes!K:K)</f>
         <v>130000</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A6" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="10">
         <f>COUNTA(_xlfn.UNIQUE(Employes!E:E))-1</f>
         <v>5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9216,20 +8735,82 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BECCEC7-2499-4969-8C4A-4F59A08AA981}">
+  <dimension ref="A3:B8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="18.53125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.59765625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A3" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="B3" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A4" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A8" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="B8">
+        <v>99</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0955E6D9-B0A9-4AB0-B598-26711973A248}">
   <dimension ref="A3:B8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18.53125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.06640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.06640625" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="6" t="s">
         <v>217</v>
       </c>
     </row>
@@ -9237,7 +8818,7 @@
       <c r="A4" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="6">
         <v>92037.037037037036</v>
       </c>
     </row>
@@ -9245,7 +8826,7 @@
       <c r="A5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="6">
         <v>85454.545454545456</v>
       </c>
     </row>
@@ -9253,7 +8834,7 @@
       <c r="A6" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="6">
         <v>89090.909090909088</v>
       </c>
     </row>
@@ -9261,7 +8842,7 @@
       <c r="A7" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="6">
         <v>80714.28571428571</v>
       </c>
     </row>
@@ -9269,7 +8850,7 @@
       <c r="A8" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="6">
         <v>86717.171717171717</v>
       </c>
     </row>
@@ -9299,7 +8880,7 @@
       <c r="A4" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4">
         <v>47</v>
       </c>
     </row>
@@ -9307,7 +8888,7 @@
       <c r="A5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5">
         <v>52</v>
       </c>
     </row>
@@ -9315,7 +8896,7 @@
       <c r="A6" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6">
         <v>99</v>
       </c>
     </row>
@@ -9345,7 +8926,7 @@
       <c r="A4" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4">
         <v>11</v>
       </c>
     </row>
@@ -9353,7 +8934,7 @@
       <c r="A5" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5">
         <v>16</v>
       </c>
     </row>
@@ -9361,7 +8942,7 @@
       <c r="A6" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6">
         <v>22</v>
       </c>
     </row>
@@ -9369,7 +8950,7 @@
       <c r="A7" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7">
         <v>21</v>
       </c>
     </row>
@@ -9377,7 +8958,7 @@
       <c r="A8" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8">
         <v>13</v>
       </c>
     </row>
@@ -9385,7 +8966,7 @@
       <c r="A9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9">
         <v>16</v>
       </c>
     </row>
@@ -9393,7 +8974,7 @@
       <c r="A10" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="B10" s="6">
+      <c r="B10">
         <v>99</v>
       </c>
     </row>

</xml_diff>